<commit_message>
Adds simple example using captest class
</commit_message>
<xml_diff>
--- a/docs/examples/data/column_groups.xlsx
+++ b/docs/examples/data/column_groups.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Example Project_Elkor Production Meter_Elkor Production Meter, KW_kW</t>
   </si>
   <si>
-    <t xml:space="preserve">wind</t>
+    <t xml:space="preserve">wind_speed</t>
   </si>
   <si>
     <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), WindSpeed_mph</t>
@@ -173,8 +173,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -190,130 +194,236 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="104.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="104.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adds a bifacial captest with CapTest class example
- Also removes the units from the example data and column groups
</commit_message>
<xml_diff>
--- a/docs/examples/data/column_groups.xlsx
+++ b/docs/examples/data/column_groups.xlsx
@@ -22,82 +22,82 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
+    <t xml:space="preserve">temp_bom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Temp1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Temp1</t>
+  </si>
+  <si>
     <t xml:space="preserve">irr_ghi</t>
   </si>
   <si>
-    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Sun2_W/m^2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Sun2_W/m^2</t>
+    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Sun2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Sun2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">temp_amb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), TempF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), TempF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real_pwr_inv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 1_Inverter 1, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 2_Inverter 2, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 3_Inverter 3, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 4_Inverter 4, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 5_Inverter 5, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 6_Inverter 6, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 7_Inverter 7, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Inverter 8_Inverter 8, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real_pwr_mtr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Elkor Production Meter_Elkor Production Meter, KW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wind_speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), WindSpeed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), WindSpeed</t>
   </si>
   <si>
     <t xml:space="preserve">irr_poa</t>
   </si>
   <si>
-    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Sun_W/m^2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Sun_W/m^2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">temp_amb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Temp1_çF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Temp1_çF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">temp_bom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), TempF_çF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), TempF_çF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real_pwr_inv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 1_Inverter 1, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 2_Inverter 2, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 3_Inverter 3, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 4_Inverter 4, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 5_Inverter 5, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 6_Inverter 6, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 7_Inverter 7, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Inverter 8_Inverter 8, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real_pwr_mtr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Elkor Production Meter_Elkor Production Meter, KW_kW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wind_speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), WindSpeed_mph</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), WindSpeed_mph</t>
+    <t xml:space="preserve">Example Project_Weather Station 1 (Standard w/ POA GHI)_Weather Station 1 (Standard w/ POA GHI), Sun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example Project_Weather Station 2 (Standard with POA GHI)_Weather Station 2 (Standard with POA GHI), Sun</t>
   </si>
 </sst>
 </file>
@@ -110,7 +110,7 @@
   <fonts count="4">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -178,7 +178,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -195,9 +195,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="LibreOffice">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -205,46 +205,46 @@
         <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -252,25 +252,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -288,12 +321,48 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -305,22 +374,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1048576"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="104.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>2</v>
       </c>
     </row>
@@ -328,12 +398,12 @@
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="0" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="0" t="s">
         <v>5</v>
       </c>
     </row>
@@ -341,12 +411,12 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="0" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="0" t="s">
         <v>8</v>
       </c>
     </row>
@@ -354,79 +424,82 @@
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="0" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="1"/>
+      <c r="B9" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="1" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="1" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="1" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="1" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="1" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="0" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="B16" s="0" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="0" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="0" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="0" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>